<commit_message>
fix: tira receita corrente menor que 2k e maior que 60k
</commit_message>
<xml_diff>
--- a/base_datas/crescimento_medio_receita_porte.xlsx
+++ b/base_datas/crescimento_medio_receita_porte.xlsx
@@ -373,7 +373,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>334.7053469608703</v>
+        <v>334.4328208923121</v>
       </c>
     </row>
     <row r="3">
@@ -393,7 +393,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>327.7652772277014</v>
+        <v>329.0721544499773</v>
       </c>
     </row>
     <row r="5">
@@ -413,7 +413,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>311.1715834413913</v>
+        <v>311.8500917193045</v>
       </c>
     </row>
     <row r="7">

</xml_diff>